<commit_message>
Reorganize and update IBF analysis workflow
</commit_message>
<xml_diff>
--- a/data/sample/remal/Remal_ddm.xlsx
+++ b/data/sample/remal/Remal_ddm.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ibrahim\Desktop\Impact Calculated for Diff lead time\ddm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ibrahim\IBF-Analysis\data\sample\remal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C292074-F8AB-4441-B28C-FF9F093427E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C011839C-15D2-4278-AB36-C5051622975B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="185">
   <si>
     <t>Chittagong</t>
   </si>
@@ -120,21 +120,12 @@
     <t>Mehendiganj</t>
   </si>
   <si>
-    <t>Banaripara</t>
-  </si>
-  <si>
     <t xml:space="preserve">Muladi </t>
   </si>
   <si>
-    <t>Hijola</t>
-  </si>
-  <si>
     <t>Barguna</t>
   </si>
   <si>
-    <t>Borhanuddin</t>
-  </si>
-  <si>
     <t>Daulatkhan</t>
   </si>
   <si>
@@ -144,15 +135,9 @@
     <t>Tazumuddin</t>
   </si>
   <si>
-    <t>Chandpur Sodor</t>
-  </si>
-  <si>
     <t>Faridganj</t>
   </si>
   <si>
-    <t>Haimchar</t>
-  </si>
-  <si>
     <t>Hajiganj</t>
   </si>
   <si>
@@ -171,9 +156,6 @@
     <t>Sandwip</t>
   </si>
   <si>
-    <t>Cox’s Bazar Sodor</t>
-  </si>
-  <si>
     <t>Eidgaon</t>
   </si>
   <si>
@@ -198,9 +180,6 @@
     <t>Feni</t>
   </si>
   <si>
-    <t>Jhalokathi</t>
-  </si>
-  <si>
     <t>Khulna</t>
   </si>
   <si>
@@ -282,12 +261,6 @@
     <t>Tala</t>
   </si>
   <si>
-    <t>Satkhira Pourashava</t>
-  </si>
-  <si>
-    <t>Kalaroa Pourashava</t>
-  </si>
-  <si>
     <t>Sonaimuri</t>
   </si>
   <si>
@@ -315,9 +288,6 @@
     <t>Sharsha</t>
   </si>
   <si>
-    <t>Ragharpara</t>
-  </si>
-  <si>
     <t>Keshabpur</t>
   </si>
   <si>
@@ -411,9 +381,6 @@
     <t>Raw House</t>
   </si>
   <si>
-    <t>Barishal</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
@@ -601,6 +568,33 @@
   </si>
   <si>
     <t>Anowara</t>
+  </si>
+  <si>
+    <t>Barisal</t>
+  </si>
+  <si>
+    <t>Jhalokati</t>
+  </si>
+  <si>
+    <t>Cox's Bazar Sadar</t>
+  </si>
+  <si>
+    <t>Banari Para</t>
+  </si>
+  <si>
+    <t>Hizla</t>
+  </si>
+  <si>
+    <t>Burhanuddin</t>
+  </si>
+  <si>
+    <t>Chandpur Sadar</t>
+  </si>
+  <si>
+    <t>Haim Char</t>
+  </si>
+  <si>
+    <t>Bagher Para</t>
   </si>
 </sst>
 </file>
@@ -1023,13 +1017,13 @@
   <sheetData>
     <row r="1" spans="1:43" x14ac:dyDescent="0.3">
       <c r="C1" s="6" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
       <c r="G1" s="7" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
@@ -1037,42 +1031,42 @@
     </row>
     <row r="2" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B3" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1136,10 +1130,10 @@
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="C4">
         <v>50</v>
@@ -1203,7 +1197,7 @@
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
@@ -1270,10 +1264,10 @@
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B6" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1337,7 +1331,7 @@
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -1404,7 +1398,7 @@
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -1471,7 +1465,7 @@
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
@@ -1538,7 +1532,7 @@
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B10" t="s">
         <v>17</v>
@@ -1605,7 +1599,7 @@
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
@@ -1672,10 +1666,10 @@
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1739,10 +1733,10 @@
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1806,7 +1800,7 @@
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
         <v>19</v>
@@ -1873,7 +1867,7 @@
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
@@ -1940,7 +1934,7 @@
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
         <v>21</v>
@@ -2007,7 +2001,7 @@
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
         <v>22</v>
@@ -2074,10 +2068,10 @@
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B18" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -2141,10 +2135,10 @@
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B19" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -2208,10 +2202,10 @@
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B20" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -2275,10 +2269,10 @@
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>179</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -2342,7 +2336,7 @@
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B22" t="s">
         <v>24</v>
@@ -2409,10 +2403,10 @@
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -2476,10 +2470,10 @@
     </row>
     <row r="24" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>180</v>
       </c>
       <c r="C24">
         <v>52</v>
@@ -2543,7 +2537,7 @@
     </row>
     <row r="25" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B25" t="s">
         <v>25</v>
@@ -2610,7 +2604,7 @@
     </row>
     <row r="26" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B26" t="s">
         <v>23</v>
@@ -2677,10 +2671,10 @@
     </row>
     <row r="27" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B27" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -2744,10 +2738,10 @@
     </row>
     <row r="28" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -2811,10 +2805,10 @@
     </row>
     <row r="29" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>181</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -2878,10 +2872,10 @@
     </row>
     <row r="30" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -2945,10 +2939,10 @@
     </row>
     <row r="31" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -3012,10 +3006,10 @@
     </row>
     <row r="32" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -3079,10 +3073,10 @@
     </row>
     <row r="33" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -3146,10 +3140,10 @@
     </row>
     <row r="34" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -3213,10 +3207,10 @@
     </row>
     <row r="35" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>34</v>
+        <v>182</v>
       </c>
       <c r="C35">
         <v>0</v>
@@ -3280,10 +3274,10 @@
     </row>
     <row r="36" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C36">
         <v>0</v>
@@ -3347,10 +3341,10 @@
     </row>
     <row r="37" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
+        <v>183</v>
       </c>
       <c r="C37">
         <v>0</v>
@@ -3414,10 +3408,10 @@
     </row>
     <row r="38" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -3481,7 +3475,7 @@
     </row>
     <row r="39" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B39" t="s">
         <v>16</v>
@@ -3548,10 +3542,10 @@
     </row>
     <row r="40" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -3615,10 +3609,10 @@
     </row>
     <row r="41" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="C41">
         <v>0</v>
@@ -3682,10 +3676,10 @@
     </row>
     <row r="42" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -3953,7 +3947,7 @@
         <v>0</v>
       </c>
       <c r="B46" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C46">
         <v>0</v>
@@ -4020,7 +4014,7 @@
         <v>0</v>
       </c>
       <c r="B47" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C47">
         <v>0</v>
@@ -4087,7 +4081,7 @@
         <v>0</v>
       </c>
       <c r="B48" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="C48">
         <v>0</v>
@@ -4288,7 +4282,7 @@
         <v>1</v>
       </c>
       <c r="B51" t="s">
-        <v>43</v>
+        <v>178</v>
       </c>
       <c r="C51">
         <v>0</v>
@@ -4422,7 +4416,7 @@
         <v>1</v>
       </c>
       <c r="B53" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C53">
         <v>0</v>
@@ -4757,7 +4751,7 @@
         <v>1</v>
       </c>
       <c r="B58" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C58">
         <v>0</v>
@@ -4888,10 +4882,10 @@
     </row>
     <row r="60" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B60" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -4955,10 +4949,10 @@
     </row>
     <row r="61" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B61" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -5022,10 +5016,10 @@
     </row>
     <row r="62" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B62" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -5089,10 +5083,10 @@
     </row>
     <row r="63" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B63" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -5156,10 +5150,10 @@
     </row>
     <row r="64" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B64" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -5223,10 +5217,10 @@
     </row>
     <row r="65" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B65" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -5290,10 +5284,10 @@
     </row>
     <row r="66" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>52</v>
+        <v>177</v>
       </c>
       <c r="B66" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -5353,10 +5347,10 @@
     </row>
     <row r="67" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>52</v>
+        <v>177</v>
       </c>
       <c r="B67" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="C67">
         <v>45</v>
@@ -5416,10 +5410,10 @@
     </row>
     <row r="68" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>52</v>
+        <v>177</v>
       </c>
       <c r="B68" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C68">
         <v>60</v>
@@ -5479,10 +5473,10 @@
     </row>
     <row r="69" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>52</v>
+        <v>177</v>
       </c>
       <c r="B69" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -5544,10 +5538,10 @@
     </row>
     <row r="70" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B70" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C70">
         <v>0</v>
@@ -5611,10 +5605,10 @@
     </row>
     <row r="71" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B71" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C71">
         <v>0</v>
@@ -5678,10 +5672,10 @@
     </row>
     <row r="72" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B72" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C72">
         <v>0</v>
@@ -5745,10 +5739,10 @@
     </row>
     <row r="73" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B73" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="C73">
         <v>0</v>
@@ -5812,10 +5806,10 @@
     </row>
     <row r="74" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B74" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="C74">
         <v>0</v>
@@ -5879,10 +5873,10 @@
     </row>
     <row r="75" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B75" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C75">
         <v>0</v>
@@ -5946,10 +5940,10 @@
     </row>
     <row r="76" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B76" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="C76">
         <v>0</v>
@@ -6013,10 +6007,10 @@
     </row>
     <row r="77" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B77" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C77">
         <v>0</v>
@@ -6080,10 +6074,10 @@
     </row>
     <row r="78" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B78" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="C78">
         <v>0</v>
@@ -6147,10 +6141,10 @@
     </row>
     <row r="79" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B79" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C79">
         <v>0</v>
@@ -6214,10 +6208,10 @@
     </row>
     <row r="80" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B80" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="C80">
         <v>9</v>
@@ -6281,10 +6275,10 @@
     </row>
     <row r="81" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B81" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="C81">
         <v>0</v>
@@ -6348,10 +6342,10 @@
     </row>
     <row r="82" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B82" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C82">
         <v>0</v>
@@ -6415,10 +6409,10 @@
     </row>
     <row r="83" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B83" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C83">
         <v>0</v>
@@ -6482,10 +6476,10 @@
     </row>
     <row r="84" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B84" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="C84">
         <v>0</v>
@@ -6549,10 +6543,10 @@
     </row>
     <row r="85" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B85" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -6616,10 +6610,10 @@
     </row>
     <row r="86" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B86" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C86">
         <v>0</v>
@@ -6683,10 +6677,10 @@
     </row>
     <row r="87" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B87" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C87">
         <v>0</v>
@@ -6750,10 +6744,10 @@
     </row>
     <row r="88" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B88" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -6817,10 +6811,10 @@
     </row>
     <row r="89" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B89" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -6884,10 +6878,10 @@
     </row>
     <row r="90" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B90" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -6951,10 +6945,10 @@
     </row>
     <row r="91" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B91" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C91">
         <v>0</v>
@@ -7018,10 +7012,10 @@
     </row>
     <row r="92" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B92" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C92">
         <v>0</v>
@@ -7085,10 +7079,10 @@
     </row>
     <row r="93" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B93" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C93">
         <v>0</v>
@@ -7152,10 +7146,10 @@
     </row>
     <row r="94" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B94" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="C94">
         <v>0</v>
@@ -7215,10 +7209,10 @@
     </row>
     <row r="95" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B95" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C95">
         <v>0</v>
@@ -7278,10 +7272,10 @@
     </row>
     <row r="96" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B96" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="C96">
         <v>60</v>
@@ -7341,10 +7335,10 @@
     </row>
     <row r="97" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B97" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="C97">
         <v>0</v>
@@ -7408,10 +7402,10 @@
     </row>
     <row r="98" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B98" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C98">
         <v>0</v>
@@ -7473,10 +7467,10 @@
     </row>
     <row r="99" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B99" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C99">
         <v>0</v>
@@ -7534,10 +7528,10 @@
     </row>
     <row r="100" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B100" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="C100">
         <v>301</v>
@@ -7599,10 +7593,10 @@
     </row>
     <row r="101" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B101" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C101">
         <v>0</v>
@@ -7666,10 +7660,10 @@
     </row>
     <row r="102" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B102" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="C102">
         <v>966</v>
@@ -7733,10 +7727,10 @@
     </row>
     <row r="103" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B103" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C103">
         <v>0</v>
@@ -7800,10 +7794,10 @@
     </row>
     <row r="104" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B104" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C104">
         <v>0</v>
@@ -7867,10 +7861,10 @@
     </row>
     <row r="105" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B105" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="C105">
         <v>0</v>
@@ -7934,10 +7928,10 @@
     </row>
     <row r="106" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B106" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="C106">
         <v>25</v>
@@ -8001,10 +7995,10 @@
     </row>
     <row r="107" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B107" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C107">
         <v>750</v>
@@ -8068,10 +8062,10 @@
     </row>
     <row r="108" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B108" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C108">
         <v>0</v>
@@ -8135,10 +8129,10 @@
     </row>
     <row r="109" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B109" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -8202,10 +8196,10 @@
     </row>
     <row r="110" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B110" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C110">
         <v>0</v>
@@ -8269,10 +8263,10 @@
     </row>
     <row r="111" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B111" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -8336,10 +8330,10 @@
     </row>
     <row r="112" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B112" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C112">
         <v>0</v>
@@ -8403,10 +8397,10 @@
     </row>
     <row r="113" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B113" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="C113">
         <v>1</v>
@@ -8470,10 +8464,10 @@
     </row>
     <row r="114" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B114" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C114">
         <v>0</v>
@@ -8537,10 +8531,10 @@
     </row>
     <row r="115" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B115" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C115">
         <v>2</v>
@@ -8604,10 +8598,10 @@
     </row>
     <row r="116" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B116" t="s">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="C116">
         <v>0</v>
@@ -8671,10 +8665,10 @@
     </row>
     <row r="117" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B117" t="s">
-        <v>81</v>
+        <v>159</v>
       </c>
       <c r="C117">
         <v>0</v>
@@ -8738,10 +8732,10 @@
     </row>
     <row r="118" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B118" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="C118">
         <v>0</v>
@@ -8805,10 +8799,10 @@
     </row>
     <row r="119" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B119" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="C119">
         <v>0</v>
@@ -8872,10 +8866,10 @@
     </row>
     <row r="120" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B120" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C120">
         <v>0</v>
@@ -8939,10 +8933,10 @@
     </row>
     <row r="121" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B121" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="C121">
         <v>0</v>
@@ -9006,10 +9000,10 @@
     </row>
     <row r="122" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B122" t="s">
-        <v>91</v>
+        <v>184</v>
       </c>
       <c r="C122">
         <v>0</v>
@@ -9073,10 +9067,10 @@
     </row>
     <row r="123" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B123" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="C123">
         <v>0</v>
@@ -9140,10 +9134,10 @@
     </row>
     <row r="124" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B124" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C124">
         <v>0</v>
@@ -9207,10 +9201,10 @@
     </row>
     <row r="125" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B125" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="C125">
         <v>0</v>
@@ -9274,10 +9268,10 @@
     </row>
     <row r="126" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B126" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="C126">
         <v>0</v>
@@ -9341,10 +9335,10 @@
     </row>
     <row r="127" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B127" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="C127">
         <v>0</v>
@@ -9408,10 +9402,10 @@
     </row>
     <row r="128" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B128" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="C128">
         <v>0</v>
@@ -9475,10 +9469,10 @@
     </row>
     <row r="129" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B129" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="C129">
         <v>0</v>
@@ -9542,10 +9536,10 @@
     </row>
     <row r="130" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B130" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C130">
         <v>0</v>
@@ -9609,10 +9603,10 @@
     </row>
     <row r="131" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B131" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="C131">
         <v>0</v>
@@ -9676,7 +9670,7 @@
     </row>
     <row r="132" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B132" t="s">
         <v>5</v>
@@ -9743,10 +9737,10 @@
     </row>
     <row r="133" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B133" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="C133">
         <v>0</v>
@@ -9810,10 +9804,10 @@
     </row>
     <row r="134" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B134" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -9874,10 +9868,10 @@
     </row>
     <row r="135" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B135" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="C135">
         <v>0</v>
@@ -9941,10 +9935,10 @@
     </row>
     <row r="136" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B136" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C136">
         <v>0</v>
@@ -10008,10 +10002,10 @@
     </row>
     <row r="137" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B137" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="C137">
         <v>0</v>
@@ -10075,10 +10069,10 @@
     </row>
     <row r="138" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B138" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -10142,10 +10136,10 @@
     </row>
     <row r="139" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B139" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C139">
         <v>1</v>
@@ -10209,10 +10203,10 @@
     </row>
     <row r="140" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B140" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C140">
         <v>0</v>
@@ -10276,10 +10270,10 @@
     </row>
     <row r="141" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B141" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="C141">
         <v>0</v>
@@ -10343,10 +10337,10 @@
     </row>
     <row r="142" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B142" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C142">
         <v>0</v>
@@ -10410,10 +10404,10 @@
     </row>
     <row r="143" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B143" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="C143">
         <v>0</v>
@@ -10477,10 +10471,10 @@
     </row>
     <row r="144" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B144" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C144">
         <v>0</v>
@@ -10544,10 +10538,10 @@
     </row>
     <row r="145" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B145" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="C145">
         <v>0</v>
@@ -10611,10 +10605,10 @@
     </row>
     <row r="146" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B146" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C146">
         <v>0</v>
@@ -10678,10 +10672,10 @@
     </row>
     <row r="147" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B147" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="C147">
         <v>0</v>
@@ -10745,10 +10739,10 @@
     </row>
     <row r="148" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B148" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="C148">
         <v>0</v>
@@ -10812,10 +10806,10 @@
     </row>
     <row r="149" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B149" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C149">
         <v>0</v>
@@ -10879,10 +10873,10 @@
     </row>
     <row r="150" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B150" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C150">
         <v>0</v>
@@ -10946,10 +10940,10 @@
     </row>
     <row r="151" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B151" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C151">
         <v>0</v>
@@ -11013,10 +11007,10 @@
     </row>
     <row r="152" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B152" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="C152">
         <v>0</v>
@@ -11080,10 +11074,10 @@
     </row>
     <row r="153" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B153" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="C153">
         <v>0</v>
@@ -11147,10 +11141,10 @@
     </row>
     <row r="154" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B154" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="C154">
         <v>0</v>
@@ -11214,10 +11208,10 @@
     </row>
     <row r="155" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B155" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C155">
         <v>0</v>
@@ -11281,10 +11275,10 @@
     </row>
     <row r="156" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B156" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="C156">
         <v>0</v>
@@ -11397,50 +11391,50 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C1" s="8" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="D1" s="8"/>
       <c r="E1" s="9" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="F1" s="9"/>
       <c r="G1" s="10" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="H1" s="10"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" t="s">
         <v>116</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>117</v>
       </c>
-      <c r="C2" t="s">
-        <v>127</v>
-      </c>
-      <c r="D2" t="s">
-        <v>128</v>
-      </c>
       <c r="E2" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="F2" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B3" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="C3" s="1">
         <v>77</v>
@@ -11465,10 +11459,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="C4" s="1">
         <v>94.64</v>
@@ -11493,7 +11487,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
@@ -11521,10 +11515,10 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B6" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
@@ -11549,7 +11543,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -11577,7 +11571,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -11605,7 +11599,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
@@ -11633,7 +11627,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B10" t="s">
         <v>17</v>
@@ -11661,7 +11655,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
@@ -11689,10 +11683,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="C12" s="1">
         <v>673.7</v>
@@ -11717,10 +11711,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="C13" s="1">
         <v>571.70000000000005</v>
@@ -11745,7 +11739,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
         <v>19</v>
@@ -11773,7 +11767,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
@@ -11801,7 +11795,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
         <v>21</v>
@@ -11829,7 +11823,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
         <v>22</v>
@@ -11857,10 +11851,10 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B18" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="C18" s="1">
         <v>93</v>
@@ -11885,10 +11879,10 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B19" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="C19" s="1">
         <v>150</v>
@@ -11913,10 +11907,10 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B20" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="C20" s="1">
         <v>0</v>
@@ -11941,10 +11935,10 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>179</v>
       </c>
       <c r="C21" s="1">
         <v>47.8</v>
@@ -11969,7 +11963,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B22" t="s">
         <v>24</v>
@@ -11997,10 +11991,10 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C23" s="1">
         <v>242.5</v>
@@ -12025,10 +12019,10 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>180</v>
       </c>
       <c r="C24" s="1">
         <v>296</v>
@@ -12053,7 +12047,7 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B25" t="s">
         <v>25</v>
@@ -12081,7 +12075,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B26" t="s">
         <v>23</v>
@@ -12109,10 +12103,10 @@
     </row>
     <row r="27" spans="1:8" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="B27" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="C27" s="1">
         <v>143</v>
@@ -12137,10 +12131,10 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="C28" s="1">
         <v>0</v>
@@ -12165,10 +12159,10 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>181</v>
       </c>
       <c r="C29" s="1">
         <v>11</v>
@@ -12193,10 +12187,10 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C30" s="1">
         <v>0</v>
@@ -12221,10 +12215,10 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C31" s="1">
         <v>0</v>
@@ -12249,10 +12243,10 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C32" s="1">
         <v>320</v>
@@ -12277,10 +12271,10 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="C33" s="1">
         <v>11060</v>
@@ -12305,10 +12299,10 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="C34" s="1">
         <v>10</v>
@@ -12333,10 +12327,10 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>34</v>
+        <v>182</v>
       </c>
       <c r="C35" s="1">
         <v>12.41</v>
@@ -12361,10 +12355,10 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C36" s="1">
         <v>14.25</v>
@@ -12389,10 +12383,10 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
+        <v>183</v>
       </c>
       <c r="C37" s="1">
         <v>16.899999999999999</v>
@@ -12417,10 +12411,10 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C38" s="1">
         <v>0</v>
@@ -12445,7 +12439,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B39" t="s">
         <v>16</v>
@@ -12473,10 +12467,10 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="C40" s="1">
         <v>10.16</v>
@@ -12501,10 +12495,10 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="C41" s="1">
         <v>4.28</v>
@@ -12529,10 +12523,10 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C42" s="1">
         <v>0</v>
@@ -12644,7 +12638,7 @@
         <v>0</v>
       </c>
       <c r="B46" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C46" s="1">
         <v>0</v>
@@ -12672,7 +12666,7 @@
         <v>0</v>
       </c>
       <c r="B47" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C47" s="1">
         <v>0</v>
@@ -12700,7 +12694,7 @@
         <v>0</v>
       </c>
       <c r="B48" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="C48" s="1">
         <v>0</v>
@@ -12784,7 +12778,7 @@
         <v>1</v>
       </c>
       <c r="B51" t="s">
-        <v>43</v>
+        <v>178</v>
       </c>
       <c r="C51" s="1">
         <v>0</v>
@@ -12840,7 +12834,7 @@
         <v>1</v>
       </c>
       <c r="B53" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C53" s="1">
         <v>0</v>
@@ -12980,7 +12974,7 @@
         <v>1</v>
       </c>
       <c r="B58" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C58" s="1">
         <v>0</v>
@@ -13033,10 +13027,10 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B60" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C60" s="1">
         <v>0</v>
@@ -13061,10 +13055,10 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B61" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C61" s="1">
         <v>0</v>
@@ -13089,10 +13083,10 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B62" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="C62" s="1">
         <v>0</v>
@@ -13117,10 +13111,10 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B63" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C63" s="1">
         <v>0</v>
@@ -13145,10 +13139,10 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B64" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="C64" s="1">
         <v>0</v>
@@ -13173,10 +13167,10 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B65" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C65" s="1">
         <v>0</v>
@@ -13201,10 +13195,10 @@
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>52</v>
+        <v>177</v>
       </c>
       <c r="B66" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="C66" s="1">
         <v>22</v>
@@ -13229,10 +13223,10 @@
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>52</v>
+        <v>177</v>
       </c>
       <c r="B67" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="D67" s="1">
         <v>0</v>
@@ -13254,10 +13248,10 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>52</v>
+        <v>177</v>
       </c>
       <c r="B68" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C68" s="1">
         <v>41</v>
@@ -13282,10 +13276,10 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>52</v>
+        <v>177</v>
       </c>
       <c r="B69" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C69" s="1">
         <v>123</v>
@@ -13310,10 +13304,10 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B70" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C70" s="1">
         <v>5</v>
@@ -13338,10 +13332,10 @@
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B71" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C71" s="1">
         <v>74</v>
@@ -13366,10 +13360,10 @@
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B72" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C72" s="1">
         <v>70.150000000000006</v>
@@ -13394,10 +13388,10 @@
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B73" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="C73" s="1">
         <v>575</v>
@@ -13422,10 +13416,10 @@
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B74" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="C74" s="1">
         <v>0</v>
@@ -13450,10 +13444,10 @@
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B75" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C75" s="1">
         <v>0</v>
@@ -13478,10 +13472,10 @@
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B76" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="C76" s="1">
         <v>3</v>
@@ -13506,10 +13500,10 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B77" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C77" s="1">
         <v>4381</v>
@@ -13534,10 +13528,10 @@
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B78" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="C78" s="1">
         <v>0</v>
@@ -13562,10 +13556,10 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B79" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C79" s="1">
         <v>0</v>
@@ -13590,10 +13584,10 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B80" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="C80" s="1">
         <v>0</v>
@@ -13618,10 +13612,10 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B81" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="C81" s="1">
         <v>0</v>
@@ -13646,10 +13640,10 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B82" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C82" s="1">
         <v>0</v>
@@ -13674,10 +13668,10 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B83" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C83" s="1">
         <v>0</v>
@@ -13702,10 +13696,10 @@
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B84" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="C84" s="1">
         <v>0</v>
@@ -13730,10 +13724,10 @@
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B85" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="C85" s="1">
         <v>86.5</v>
@@ -13758,10 +13752,10 @@
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B86" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C86" s="1">
         <v>80</v>
@@ -13786,10 +13780,10 @@
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B87" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C87" s="1">
         <v>0</v>
@@ -13814,10 +13808,10 @@
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B88" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C88" s="1">
         <v>0</v>
@@ -13842,10 +13836,10 @@
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B89" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="C89" s="1">
         <v>1242</v>
@@ -13870,10 +13864,10 @@
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B90" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="C90" s="1">
         <v>0</v>
@@ -13898,10 +13892,10 @@
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B91" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C91" s="1">
         <v>0</v>
@@ -13926,10 +13920,10 @@
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B92" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C92" s="1">
         <v>0</v>
@@ -13954,10 +13948,10 @@
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B93" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C93" s="1">
         <v>0</v>
@@ -13982,10 +13976,10 @@
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B94" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="C94" s="1">
         <v>0</v>
@@ -14010,10 +14004,10 @@
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B95" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C95" s="1">
         <v>103</v>
@@ -14035,10 +14029,10 @@
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B96" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="C96" s="1">
         <v>80</v>
@@ -14063,10 +14057,10 @@
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B97" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="C97" s="1">
         <v>165</v>
@@ -14091,10 +14085,10 @@
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B98" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C98" s="1">
         <v>255</v>
@@ -14119,10 +14113,10 @@
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B99" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C99" s="1">
         <v>885</v>
@@ -14144,10 +14138,10 @@
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B100" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="D100" s="1">
         <v>0</v>
@@ -14169,10 +14163,10 @@
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B101" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C101" s="1">
         <v>180</v>
@@ -14197,10 +14191,10 @@
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B102" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="C102" s="1">
         <v>480</v>
@@ -14225,10 +14219,10 @@
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B103" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C103" s="1">
         <v>390</v>
@@ -14253,10 +14247,10 @@
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B104" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C104" s="1">
         <v>1</v>
@@ -14281,10 +14275,10 @@
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B105" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="C105" s="1">
         <v>1744</v>
@@ -14309,10 +14303,10 @@
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B106" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="C106" s="1">
         <v>2</v>
@@ -14337,10 +14331,10 @@
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B107" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C107" s="1">
         <v>0</v>
@@ -14365,10 +14359,10 @@
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="B108" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C108" s="1">
         <v>194</v>
@@ -14393,10 +14387,10 @@
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B109" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="C109" s="1">
         <v>0</v>
@@ -14421,10 +14415,10 @@
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B110" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C110" s="1">
         <v>0</v>
@@ -14449,10 +14443,10 @@
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B111" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="C111" s="1">
         <v>0</v>
@@ -14477,10 +14471,10 @@
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B112" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C112" s="1">
         <v>0</v>
@@ -14505,10 +14499,10 @@
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B113" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="C113" s="1">
         <v>10</v>
@@ -14533,10 +14527,10 @@
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B114" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C114" s="1">
         <v>0</v>
@@ -14561,10 +14555,10 @@
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B115" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C115" s="1">
         <v>0</v>
@@ -14589,10 +14583,10 @@
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B116" t="s">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="C116" s="1">
         <v>0</v>
@@ -14617,10 +14611,10 @@
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B117" t="s">
-        <v>81</v>
+        <v>159</v>
       </c>
       <c r="C117" s="1">
         <v>0</v>
@@ -14645,10 +14639,10 @@
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B118" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="C118" s="1">
         <v>0</v>
@@ -14673,10 +14667,10 @@
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B119" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="C119" s="1">
         <v>0</v>
@@ -14701,10 +14695,10 @@
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B120" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C120" s="1">
         <v>0</v>
@@ -14729,10 +14723,10 @@
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B121" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="C121" s="1">
         <v>0</v>
@@ -14757,10 +14751,10 @@
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B122" t="s">
-        <v>91</v>
+        <v>184</v>
       </c>
       <c r="C122" s="1">
         <v>0</v>
@@ -14785,10 +14779,10 @@
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B123" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="C123" s="1">
         <v>0</v>
@@ -14813,10 +14807,10 @@
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B124" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C124" s="1">
         <v>0</v>
@@ -14841,10 +14835,10 @@
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B125" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="C125" s="1">
         <v>0</v>
@@ -14869,10 +14863,10 @@
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B126" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="C126" s="1">
         <v>0</v>
@@ -14897,10 +14891,10 @@
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B127" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="C127" s="1">
         <v>0</v>
@@ -14925,10 +14919,10 @@
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B128" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="C128" s="1">
         <v>0</v>
@@ -14953,10 +14947,10 @@
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B129" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="C129" s="1">
         <v>0</v>
@@ -14981,10 +14975,10 @@
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B130" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C130" s="1">
         <v>420</v>
@@ -15009,10 +15003,10 @@
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B131" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="C131" s="1">
         <v>0</v>
@@ -15037,7 +15031,7 @@
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B132" t="s">
         <v>5</v>
@@ -15065,10 +15059,10 @@
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B133" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="C133" s="1">
         <v>50</v>
@@ -15093,10 +15087,10 @@
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B134" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="C134" s="1">
         <v>0</v>
@@ -15121,10 +15115,10 @@
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B135" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="C135" s="1">
         <v>0</v>
@@ -15149,10 +15143,10 @@
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B136" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C136" s="1">
         <v>20</v>
@@ -15177,10 +15171,10 @@
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B137" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="C137" s="1">
         <v>0</v>
@@ -15205,10 +15199,10 @@
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B138" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="C138" s="1">
         <v>0</v>
@@ -15233,10 +15227,10 @@
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B139" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="C139" s="1">
         <v>5</v>
@@ -15261,10 +15255,10 @@
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B140" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="C140" s="1">
         <v>2</v>
@@ -15289,10 +15283,10 @@
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B141" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="C141" s="1">
         <v>5</v>
@@ -15317,10 +15311,10 @@
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B142" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C142" s="1">
         <v>1</v>
@@ -15345,10 +15339,10 @@
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B143" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="C143" s="1">
         <v>5</v>
@@ -15373,10 +15367,10 @@
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B144" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C144" s="1">
         <v>2</v>
@@ -15401,10 +15395,10 @@
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B145" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="C145" s="1">
         <v>0</v>
@@ -15429,10 +15423,10 @@
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B146" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C146" s="1">
         <v>1</v>
@@ -15457,10 +15451,10 @@
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B147" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="C147" s="1">
         <v>0</v>
@@ -15485,10 +15479,10 @@
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B148" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="C148" s="1">
         <v>0</v>
@@ -15513,10 +15507,10 @@
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B149" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C149" s="1">
         <v>1</v>
@@ -15541,10 +15535,10 @@
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B150" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C150" s="1">
         <v>1</v>
@@ -15569,10 +15563,10 @@
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B151" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C151" s="1">
         <v>0</v>
@@ -15597,10 +15591,10 @@
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B152" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="C152" s="1">
         <v>1</v>
@@ -15625,10 +15619,10 @@
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B153" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="C153" s="1">
         <v>0</v>
@@ -15653,10 +15647,10 @@
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B154" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="C154" s="1">
         <v>0</v>
@@ -15681,10 +15675,10 @@
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B155" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C155" s="1">
         <v>0</v>
@@ -15709,10 +15703,10 @@
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B156" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="C156" s="1">
         <v>0</v>

</xml_diff>